<commit_message>
Deleted redundant figures and simplified climate annotation code
</commit_message>
<xml_diff>
--- a/Demographic analysis sites.xlsx
+++ b/Demographic analysis sites.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brandon Nguyen\Documents\Independent study\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3410420-E67B-454A-8E4E-AB546EE7828A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FC958C-F9B1-4866-BEA8-95808DACEC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="147">
   <si>
     <t>Site</t>
   </si>
@@ -462,6 +462,9 @@
   </si>
   <si>
     <t>Nesje and Dahl 2001</t>
+  </si>
+  <si>
+    <t>8.2k</t>
   </si>
 </sst>
 </file>
@@ -10389,9 +10392,7 @@
       <c r="F14" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>118</v>
-      </c>
+      <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
@@ -10630,8 +10631,8 @@
       <c r="E25" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F25" s="2">
-        <v>8.1999999999999993</v>
+      <c r="F25" s="2" t="s">
+        <v>146</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>118</v>

</xml_diff>